<commit_message>
change plantilal cotizacion inicial calculdora
</commit_message>
<xml_diff>
--- a/public/assets/templates/PLANTILLA_COTIZACION_INICIAL_CALCULADORA.xlsx
+++ b/public/assets/templates/PLANTILLA_COTIZACION_INICIAL_CALCULADORA.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\OneDrive\Desktop\Proyectos\Probusiness\probusiness_intranetv2_back\public\assets\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3D28B47-ECD5-45F7-AF7B-3A5AE83342A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C38E9FF6-1926-4762-ADE6-73692AC2E649}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="735" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="132">
   <si>
     <t>VALOR UNITARIO</t>
   </si>
@@ -172,21 +172,6 @@
     <t># ITEM</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Todos los pagos se realizan en dólares. </t>
-  </si>
-  <si>
-    <t>3. No somos responsables de retraso del proveedor para entregar la carga.</t>
-  </si>
-  <si>
-    <t>5.Los pagos realizados fuera de fecha están sujetos a un recargo de S/.30 por día.</t>
-  </si>
-  <si>
-    <t>9.No hay opción de reembolso.</t>
-  </si>
-  <si>
-    <t>6.Se procederá a cobrar S/.30 x día de almacenaje si el cliente no recoge su pedido en el plazo acordado.</t>
-  </si>
-  <si>
     <t>se procederá a realizar las acciones legales del caso.</t>
   </si>
   <si>
@@ -196,70 +181,15 @@
     <t xml:space="preserve"> No se aceptan marcas con medidas  de frontera. </t>
   </si>
   <si>
-    <t>2.Todas las marcas de los productos deben ser verificadas por el cliente,</t>
-  </si>
-  <si>
     <t>En caso contrario, asumirá el costo de  almacenaje $30 y será embarcado en la próxima salida.</t>
   </si>
   <si>
-    <t>4. La carga deberá llegar al almacén –Yiwu en el rango de fecha indicado por su asesor.</t>
-  </si>
-  <si>
-    <t>7.Los envíos a provincia se realizan a través de la agencia Marvisur o Shalom, con previo pago de flete interno.</t>
-  </si>
-  <si>
     <t>Costo: desde s/20.00</t>
   </si>
   <si>
     <t>coordinador  logístico la tarifa.</t>
   </si>
   <si>
-    <t>8. Las cargas mayores a 200 kg x bulto tendrán un costo adicional por manipuleo, consultar con el</t>
-  </si>
-  <si>
-    <t>11. El costo por metro cubico incluye: Flete – Ag. Aduana – Costos en destino.</t>
-  </si>
-  <si>
-    <r>
-      <t>13.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Calibri Light"/>
-        <family val="2"/>
-        <scheme val="major"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri Light"/>
-        <family val="2"/>
-        <scheme val="major"/>
-      </rPr>
-      <t>Los documentos de importación deber ser entregados a tiempo, de lo contrario, el participante no tendrá opción</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">14.En caso el cliente esté importando una carga que no sea legal y la empresa Pro Business se vea perjudicada, </t>
-  </si>
-  <si>
-    <t xml:space="preserve">15.El cliente estará sujeto a pagar mayor el ad- valorem en caso aduanas aplique cambios de partida. </t>
-  </si>
-  <si>
-    <t>16.Si el cliente no paga los tributos o gastos administrativos de su cotización, Pro Business será dueño total de la carga.</t>
-  </si>
-  <si>
-    <t>17.Los ajustes de valor que aplique la aduana serán asumidos por el cliente.</t>
-  </si>
-  <si>
-    <t>18.No somos responsable de las mermas o faltante de la carga (entregamos su pedido tal cual el proveedor envío).</t>
-  </si>
-  <si>
     <t>VALOR ZAPATILLAS</t>
   </si>
   <si>
@@ -291,12 +221,6 @@
   </si>
   <si>
     <t>NUEVO</t>
-  </si>
-  <si>
-    <t>20.Las mercancías son declaradas a nombre de la empresa Grupo Pro Business.</t>
-  </si>
-  <si>
-    <t>21.Se emitirá comprobante (boleta o Factura) de su importación en base a la estrategia de declaración realizada.</t>
   </si>
   <si>
     <t>TOTAL CBM</t>
@@ -580,27 +504,9 @@
     <t>RESUMEN DE COSTOS UNITARIOS</t>
   </si>
   <si>
-    <t>12.No se aceptan productos restringido que no cuenten con permiso.</t>
-  </si>
-  <si>
     <t>de acogerse a un beneficio arancelario (C.O) o pueda tener perdida en aduanas por informacion incompleta.</t>
   </si>
   <si>
-    <t>19.La fecha de entrega es aproximada, está sujeto a variaciones de linea naviera o aduanas.</t>
-  </si>
-  <si>
-    <t>10. Si el cliente quiere cambiar la salida de su carga debera informar 4 día antes de la fecha de cierre.</t>
-  </si>
-  <si>
-    <t>22. El cliente tendra un plazo de 24 horas despues de la entrega para presentar algun tipo de reclamo.</t>
-  </si>
-  <si>
-    <t>23. La factura o boleta se emitirá con base al valor CIF de la cotización final.</t>
-  </si>
-  <si>
-    <t>24. Concepto no facturable: Advalorem, Percepción, Anti-Dumping o Gestión de Compra</t>
-  </si>
-  <si>
     <t>N PROVEEDOR</t>
   </si>
   <si>
@@ -647,6 +553,103 @@
   </si>
   <si>
     <t>Deposito a nuestra cuenta bancaria para pagar impuestos ante Aduanas antes de llegar a puerto (Callao)</t>
+  </si>
+  <si>
+    <t>2.Los productos que tengan un peso mayor o igual a 100 kgs se le realizará el recargo por el uso de montacarga.</t>
+  </si>
+  <si>
+    <t>3.Todas las marcas de los productos deben ser verificadas por el cliente,</t>
+  </si>
+  <si>
+    <t>4. No somos responsables de retraso del proveedor para entregar la carga.</t>
+  </si>
+  <si>
+    <t>5. La carga deberá llegar al almacén –Yiwu en el rango de fecha indicado por su asesor.</t>
+  </si>
+  <si>
+    <t>6.Los pagos realizados fuera de fecha están sujetos a un recargo de S/.30 por día.</t>
+  </si>
+  <si>
+    <t>7.Se procederá a cobrar S/.30 x día de almacenaje si el cliente no recoge su pedido en el plazo acordado.</t>
+  </si>
+  <si>
+    <t>8.Los envíos a provincia se realizan a través de la agencia Marvisur o Shalom, con previo pago de flete interno.</t>
+  </si>
+  <si>
+    <t>10.No hay opción de reembolso.</t>
+  </si>
+  <si>
+    <t>11. Si el cliente quiere cambiar la salida de su carga debera informar 4 día antes de la fecha de cierre.</t>
+  </si>
+  <si>
+    <t>1. La cotización tiene una vida útil de 48 horas hábiles</t>
+  </si>
+  <si>
+    <t>9. Las cargas mayores a 100 kg x bulto tendrán un costo adicional por manipuleo, consultar con el</t>
+  </si>
+  <si>
+    <t>12. El costo por metro cubico incluye: Flete – Ag. Aduana – Costos en destino.</t>
+  </si>
+  <si>
+    <t>13.No se aceptan productos restringido que no cuenten con permiso.</t>
+  </si>
+  <si>
+    <r>
+      <t>14.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color theme="1"/>
+        <rFont val="Calibri Light"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri Light"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </rPr>
+      <t>Los documentos de importación deber ser entregados a tiempo, de lo contrario, el participante no tendrá opción</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">15.En caso el cliente esté importando una carga que no sea legal y la empresa Pro Business se vea perjudicada, </t>
+  </si>
+  <si>
+    <t xml:space="preserve">16.El cliente estará sujeto a pagar mayor el ad- valorem en caso aduanas aplique cambios de partida. </t>
+  </si>
+  <si>
+    <t>17.Si el cliente no paga los tributos o gastos administrativos de su cotización, Pro Business será dueño total de la carga.</t>
+  </si>
+  <si>
+    <t>18.Los ajustes de valor que aplique la aduana serán asumidos por el cliente.</t>
+  </si>
+  <si>
+    <t>19.No somos responsable de las mermas o faltante de la carga (entregamos su pedido tal cual el proveedor envío).</t>
+  </si>
+  <si>
+    <t>20.La fecha de entrega es aproximada, está sujeto a variaciones de linea naviera o aduanas.</t>
+  </si>
+  <si>
+    <t>21.Las mercancías son declaradas a nombre de la empresa Grupo Pro Business.</t>
+  </si>
+  <si>
+    <t>22.Se emitirá comprobante (boleta o Factura) de su importación en base a la estrategia de declaración realizada.</t>
+  </si>
+  <si>
+    <t>23. El cliente tendra un plazo de 24 horas despues de la entrega para presentar algun tipo de reclamo.</t>
+  </si>
+  <si>
+    <t>24. La factura o boleta se emitirá con base al valor CIF de la cotización final.</t>
+  </si>
+  <si>
+    <t>25. Concepto no facturable: Advalorem, Percepción, Anti-Dumping o Gestión de Compra</t>
   </si>
 </sst>
 </file>
@@ -1636,6 +1639,86 @@
     <xf numFmtId="2" fontId="31" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="36" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="38" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="8" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="172" fontId="26" fillId="11" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1666,71 +1749,20 @@
     <xf numFmtId="0" fontId="20" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="172" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="8" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="172" fontId="26" fillId="11" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="172" fontId="26" fillId="11" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="38" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="26" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="26" fillId="11" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="26" fillId="11" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="26" fillId="11" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="26" fillId="11" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="26" fillId="11" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="172" fontId="26" fillId="11" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="172" fontId="26" fillId="11" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="169" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="171" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1752,35 +1784,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="38" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="2" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="14">
@@ -2571,15 +2574,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>62</xdr:row>
-      <xdr:rowOff>79078</xdr:rowOff>
+      <xdr:colOff>89648</xdr:colOff>
+      <xdr:row>56</xdr:row>
+      <xdr:rowOff>45463</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>239621</xdr:colOff>
-      <xdr:row>94</xdr:row>
-      <xdr:rowOff>33834</xdr:rowOff>
+      <xdr:colOff>329269</xdr:colOff>
+      <xdr:row>88</xdr:row>
+      <xdr:rowOff>219</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2608,8 +2611,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="18776300"/>
-          <a:ext cx="7639885" cy="6276534"/>
+          <a:off x="89648" y="11654757"/>
+          <a:ext cx="6716621" cy="6050756"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2958,40 +2961,40 @@
     <row r="1" spans="1:11" ht="18.75" customHeight="1"/>
     <row r="2" spans="1:11" ht="18.75" customHeight="1"/>
     <row r="3" spans="1:11">
-      <c r="C3" s="125" t="s">
-        <v>121</v>
-      </c>
-      <c r="D3" s="125"/>
-      <c r="E3" s="125"/>
-      <c r="F3" s="125"/>
-      <c r="G3" s="125"/>
+      <c r="C3" s="120" t="s">
+        <v>97</v>
+      </c>
+      <c r="D3" s="120"/>
+      <c r="E3" s="120"/>
+      <c r="F3" s="120"/>
+      <c r="G3" s="120"/>
     </row>
     <row r="4" spans="1:11">
-      <c r="C4" s="125"/>
-      <c r="D4" s="125"/>
-      <c r="E4" s="125"/>
-      <c r="F4" s="125"/>
-      <c r="G4" s="125"/>
+      <c r="C4" s="120"/>
+      <c r="D4" s="120"/>
+      <c r="E4" s="120"/>
+      <c r="F4" s="120"/>
+      <c r="G4" s="120"/>
     </row>
     <row r="5" spans="1:11" ht="26.25">
-      <c r="C5" s="126" t="s">
-        <v>122</v>
-      </c>
-      <c r="D5" s="126"/>
-      <c r="E5" s="126"/>
-      <c r="F5" s="126"/>
-      <c r="G5" s="126"/>
+      <c r="C5" s="121" t="s">
+        <v>98</v>
+      </c>
+      <c r="D5" s="121"/>
+      <c r="E5" s="121"/>
+      <c r="F5" s="121"/>
+      <c r="G5" s="121"/>
     </row>
     <row r="7" spans="1:11">
-      <c r="D7" s="141" t="s">
-        <v>102</v>
-      </c>
-      <c r="E7" s="141"/>
-      <c r="F7" s="141"/>
+      <c r="D7" s="136" t="s">
+        <v>84</v>
+      </c>
+      <c r="E7" s="136"/>
+      <c r="F7" s="136"/>
     </row>
     <row r="8" spans="1:11">
       <c r="A8" s="33" t="s">
-        <v>78</v>
+        <v>62</v>
       </c>
       <c r="B8" s="47"/>
       <c r="D8" s="64" t="s">
@@ -3005,40 +3008,40 @@
       <c r="H8" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="I8" s="143">
+      <c r="I8" s="139">
         <f>+'2'!D5</f>
         <v>1</v>
       </c>
-      <c r="J8" s="143"/>
-      <c r="K8" s="143"/>
+      <c r="J8" s="139"/>
+      <c r="K8" s="139"/>
     </row>
     <row r="9" spans="1:11">
       <c r="A9" s="33" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="B9" s="47"/>
       <c r="D9" s="67" t="s">
-        <v>94</v>
-      </c>
-      <c r="E9" s="127">
+        <v>76</v>
+      </c>
+      <c r="E9" s="122">
         <f ca="1">+TODAY()</f>
-        <v>46062</v>
-      </c>
-      <c r="F9" s="128"/>
+        <v>46094</v>
+      </c>
+      <c r="F9" s="123"/>
       <c r="G9" s="31"/>
       <c r="H9" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="I9" s="144">
+      <c r="I9" s="140">
         <f>+'2'!D6</f>
         <v>23.2</v>
       </c>
-      <c r="J9" s="144"/>
-      <c r="K9" s="144"/>
+      <c r="J9" s="140"/>
+      <c r="K9" s="140"/>
     </row>
     <row r="10" spans="1:11">
       <c r="A10" s="33" t="s">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="B10" s="47"/>
       <c r="D10" s="74" t="s">
@@ -3050,7 +3053,7 @@
       <c r="F10" s="73"/>
       <c r="G10" s="31"/>
       <c r="H10" s="1" t="s">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="I10" s="80">
         <v>0</v>
@@ -3071,27 +3074,27 @@
         <v>22</v>
       </c>
       <c r="E11" s="38" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="F11" s="69"/>
       <c r="H11" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="I11" s="142">
+      <c r="I11" s="137">
         <f>+'2'!D8</f>
         <v>8.4000000000000005E-2</v>
       </c>
-      <c r="J11" s="142"/>
-      <c r="K11" s="142"/>
+      <c r="J11" s="137"/>
+      <c r="K11" s="137"/>
     </row>
     <row r="13" spans="1:11">
-      <c r="A13" s="123" t="s">
+      <c r="A13" s="138" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="123"/>
-      <c r="C13" s="123"/>
-      <c r="D13" s="123"/>
-      <c r="E13" s="123"/>
+      <c r="B13" s="138"/>
+      <c r="C13" s="138"/>
+      <c r="D13" s="138"/>
+      <c r="E13" s="138"/>
       <c r="F13" s="58"/>
       <c r="G13" s="58"/>
       <c r="H13" s="60"/>
@@ -3104,11 +3107,11 @@
       </c>
     </row>
     <row r="14" spans="1:11">
-      <c r="A14" s="115" t="s">
+      <c r="A14" s="143" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="115"/>
-      <c r="C14" s="115"/>
+      <c r="B14" s="143"/>
+      <c r="C14" s="143"/>
       <c r="D14" s="31"/>
       <c r="E14" s="31"/>
       <c r="F14" s="31"/>
@@ -3122,11 +3125,11 @@
       </c>
     </row>
     <row r="15" spans="1:11">
-      <c r="A15" s="114" t="s">
+      <c r="A15" s="142" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="114"/>
-      <c r="C15" s="114"/>
+      <c r="B15" s="142"/>
+      <c r="C15" s="142"/>
       <c r="D15" s="38"/>
       <c r="E15" s="38"/>
       <c r="F15" s="38"/>
@@ -3188,13 +3191,13 @@
       <c r="K18" s="31"/>
     </row>
     <row r="19" spans="1:12">
-      <c r="A19" s="123" t="s">
-        <v>92</v>
-      </c>
-      <c r="B19" s="123"/>
-      <c r="C19" s="123"/>
-      <c r="D19" s="123"/>
-      <c r="E19" s="123"/>
+      <c r="A19" s="138" t="s">
+        <v>74</v>
+      </c>
+      <c r="B19" s="138"/>
+      <c r="C19" s="138"/>
+      <c r="D19" s="138"/>
+      <c r="E19" s="138"/>
       <c r="F19" s="58"/>
       <c r="G19" s="58"/>
       <c r="H19" s="58"/>
@@ -3343,7 +3346,7 @@
       <c r="G26" s="38"/>
       <c r="H26" s="38"/>
       <c r="I26" s="62" t="s">
-        <v>73</v>
+        <v>57</v>
       </c>
       <c r="J26" s="46" t="e">
         <f>'2'!D37</f>
@@ -3373,13 +3376,13 @@
       </c>
     </row>
     <row r="29" spans="1:12" ht="15.75">
-      <c r="A29" s="122" t="s">
-        <v>89</v>
-      </c>
-      <c r="B29" s="122"/>
-      <c r="C29" s="122"/>
-      <c r="D29" s="122"/>
-      <c r="E29" s="122"/>
+      <c r="A29" s="150" t="s">
+        <v>71</v>
+      </c>
+      <c r="B29" s="150"/>
+      <c r="C29" s="150"/>
+      <c r="D29" s="150"/>
+      <c r="E29" s="150"/>
       <c r="F29" s="78"/>
       <c r="G29" s="78"/>
       <c r="H29" s="79"/>
@@ -3393,7 +3396,7 @@
     </row>
     <row r="30" spans="1:12">
       <c r="A30" s="31" t="s">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="B30" s="31"/>
       <c r="C30" s="31"/>
@@ -3413,7 +3416,7 @@
     </row>
     <row r="31" spans="1:12">
       <c r="A31" s="31" t="s">
-        <v>119</v>
+        <v>95</v>
       </c>
       <c r="B31" s="31"/>
       <c r="C31" s="31"/>
@@ -3432,7 +3435,7 @@
     </row>
     <row r="32" spans="1:12">
       <c r="A32" s="104" t="s">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="B32" s="31"/>
       <c r="C32" s="31"/>
@@ -3473,7 +3476,7 @@
     </row>
     <row r="34" spans="1:19">
       <c r="A34" s="33" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="B34" s="31"/>
       <c r="C34" s="31"/>
@@ -3490,13 +3493,13 @@
       <c r="K34" s="34" t="s">
         <v>35</v>
       </c>
-      <c r="M34" s="131" t="s">
-        <v>107</v>
-      </c>
-      <c r="N34" s="131"/>
-      <c r="O34" s="131"/>
-      <c r="P34" s="131"/>
-      <c r="Q34" s="131"/>
+      <c r="M34" s="126" t="s">
+        <v>89</v>
+      </c>
+      <c r="N34" s="126"/>
+      <c r="O34" s="126"/>
+      <c r="P34" s="126"/>
+      <c r="Q34" s="126"/>
     </row>
     <row r="35" spans="1:19" ht="20.25" customHeight="1">
       <c r="A35" s="33"/>
@@ -3510,73 +3513,73 @@
       <c r="I35" s="37"/>
       <c r="J35" s="37"/>
       <c r="K35" s="34"/>
-      <c r="M35" s="132"/>
-      <c r="N35" s="132"/>
-      <c r="O35" s="132"/>
-      <c r="P35" s="132"/>
-      <c r="Q35" s="132"/>
+      <c r="M35" s="127"/>
+      <c r="N35" s="127"/>
+      <c r="O35" s="127"/>
+      <c r="P35" s="127"/>
+      <c r="Q35" s="127"/>
     </row>
     <row r="36" spans="1:19" ht="15" customHeight="1">
-      <c r="A36" s="118" t="s">
-        <v>93</v>
-      </c>
-      <c r="B36" s="119"/>
-      <c r="C36" s="119"/>
-      <c r="D36" s="119"/>
-      <c r="E36" s="119"/>
-      <c r="F36" s="119"/>
-      <c r="G36" s="119"/>
-      <c r="H36" s="119"/>
-      <c r="I36" s="119"/>
-      <c r="J36" s="119"/>
-      <c r="K36" s="120"/>
-      <c r="M36" s="139" t="s">
+      <c r="A36" s="146" t="s">
+        <v>75</v>
+      </c>
+      <c r="B36" s="147"/>
+      <c r="C36" s="147"/>
+      <c r="D36" s="147"/>
+      <c r="E36" s="147"/>
+      <c r="F36" s="147"/>
+      <c r="G36" s="147"/>
+      <c r="H36" s="147"/>
+      <c r="I36" s="147"/>
+      <c r="J36" s="147"/>
+      <c r="K36" s="148"/>
+      <c r="M36" s="134" t="s">
         <v>46</v>
       </c>
-      <c r="N36" s="137" t="s">
-        <v>76</v>
-      </c>
-      <c r="O36" s="133" t="s">
-        <v>103</v>
-      </c>
-      <c r="P36" s="135" t="s">
-        <v>104</v>
-      </c>
-      <c r="Q36" s="129" t="s">
-        <v>105</v>
+      <c r="N36" s="132" t="s">
+        <v>60</v>
+      </c>
+      <c r="O36" s="128" t="s">
+        <v>85</v>
+      </c>
+      <c r="P36" s="130" t="s">
+        <v>86</v>
+      </c>
+      <c r="Q36" s="124" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="37" spans="1:19" ht="17.25" customHeight="1">
       <c r="A37" s="59" t="s">
         <v>46</v>
       </c>
-      <c r="B37" s="116" t="s">
-        <v>76</v>
-      </c>
-      <c r="C37" s="121"/>
-      <c r="D37" s="117"/>
+      <c r="B37" s="144" t="s">
+        <v>60</v>
+      </c>
+      <c r="C37" s="149"/>
+      <c r="D37" s="145"/>
       <c r="E37" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="F37" s="116" t="s">
-        <v>77</v>
-      </c>
-      <c r="G37" s="117"/>
+      <c r="F37" s="144" t="s">
+        <v>61</v>
+      </c>
+      <c r="G37" s="145"/>
       <c r="H37" s="5" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="I37" s="70" t="s">
         <v>8</v>
       </c>
-      <c r="J37" s="124" t="s">
-        <v>75</v>
-      </c>
-      <c r="K37" s="124"/>
-      <c r="M37" s="140"/>
-      <c r="N37" s="138"/>
-      <c r="O37" s="134"/>
-      <c r="P37" s="136"/>
-      <c r="Q37" s="130"/>
+      <c r="J37" s="151" t="s">
+        <v>59</v>
+      </c>
+      <c r="K37" s="151"/>
+      <c r="M37" s="135"/>
+      <c r="N37" s="133"/>
+      <c r="O37" s="129"/>
+      <c r="P37" s="131"/>
+      <c r="Q37" s="125"/>
     </row>
     <row r="38" spans="1:19" s="109" customFormat="1" ht="15.75">
       <c r="A38" s="106" t="s">
@@ -3610,19 +3613,19 @@
       <c r="I39" s="83"/>
       <c r="J39" s="71"/>
       <c r="K39" s="72"/>
-      <c r="M39" s="152" t="s">
-        <v>106</v>
-      </c>
-      <c r="N39" s="152"/>
-      <c r="O39" s="152"/>
-      <c r="P39" s="152"/>
-      <c r="Q39" s="152"/>
-      <c r="R39" s="152"/>
-      <c r="S39" s="152"/>
+      <c r="M39" s="153" t="s">
+        <v>88</v>
+      </c>
+      <c r="N39" s="153"/>
+      <c r="O39" s="153"/>
+      <c r="P39" s="153"/>
+      <c r="Q39" s="153"/>
+      <c r="R39" s="153"/>
+      <c r="S39" s="153"/>
     </row>
     <row r="40" spans="1:19" ht="18.75" customHeight="1">
       <c r="A40" s="81" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B40" s="31"/>
       <c r="C40" s="31"/>
@@ -3633,17 +3636,17 @@
       <c r="H40" s="31"/>
       <c r="I40" s="31"/>
       <c r="J40" s="31"/>
-      <c r="M40" s="152"/>
-      <c r="N40" s="152"/>
-      <c r="O40" s="152"/>
-      <c r="P40" s="152"/>
-      <c r="Q40" s="152"/>
-      <c r="R40" s="152"/>
-      <c r="S40" s="152"/>
+      <c r="M40" s="153"/>
+      <c r="N40" s="153"/>
+      <c r="O40" s="153"/>
+      <c r="P40" s="153"/>
+      <c r="Q40" s="153"/>
+      <c r="R40" s="153"/>
+      <c r="S40" s="153"/>
     </row>
     <row r="41" spans="1:19" ht="18.75">
       <c r="A41" s="82" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="B41" s="31"/>
       <c r="C41" s="31"/>
@@ -3657,7 +3660,7 @@
     </row>
     <row r="42" spans="1:19" ht="18.75">
       <c r="A42" s="82" t="s">
-        <v>85</v>
+        <v>67</v>
       </c>
       <c r="B42" s="31"/>
       <c r="C42" s="31"/>
@@ -3668,19 +3671,19 @@
       <c r="H42" s="31"/>
       <c r="I42" s="31"/>
       <c r="J42" s="31"/>
-      <c r="M42" s="153" t="s">
-        <v>123</v>
-      </c>
-      <c r="O42" s="153" t="s">
+      <c r="M42" s="113" t="s">
+        <v>99</v>
+      </c>
+      <c r="O42" s="113" t="s">
         <v>34</v>
       </c>
-      <c r="R42" s="153" t="s">
-        <v>124</v>
+      <c r="R42" s="113" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="43" spans="1:19" ht="18.75">
       <c r="A43" s="82" t="s">
-        <v>96</v>
+        <v>78</v>
       </c>
       <c r="B43" s="31"/>
       <c r="C43" s="31"/>
@@ -3691,13 +3694,13 @@
       <c r="H43" s="31"/>
       <c r="I43" s="31"/>
       <c r="J43" s="31"/>
-      <c r="N43" s="154"/>
-      <c r="O43" s="154"/>
-      <c r="P43" s="154"/>
+      <c r="N43" s="114"/>
+      <c r="O43" s="114"/>
+      <c r="P43" s="114"/>
     </row>
     <row r="44" spans="1:19" ht="18.75" customHeight="1">
       <c r="A44" s="82" t="s">
-        <v>86</v>
+        <v>68</v>
       </c>
       <c r="B44" s="31"/>
       <c r="C44" s="31"/>
@@ -3708,24 +3711,24 @@
       <c r="H44" s="31"/>
       <c r="I44" s="31"/>
       <c r="J44" s="31"/>
-      <c r="M44" s="155" t="s">
-        <v>125</v>
+      <c r="M44" s="154" t="s">
+        <v>101</v>
       </c>
       <c r="N44" s="31"/>
-      <c r="O44" s="156">
+      <c r="O44" s="152">
         <f>J14</f>
         <v>1220</v>
       </c>
       <c r="P44" s="31"/>
-      <c r="Q44" s="157" t="s">
-        <v>126</v>
-      </c>
-      <c r="R44" s="157"/>
-      <c r="S44" s="157"/>
+      <c r="Q44" s="119" t="s">
+        <v>102</v>
+      </c>
+      <c r="R44" s="119"/>
+      <c r="S44" s="119"/>
     </row>
     <row r="45" spans="1:19" ht="18.75" customHeight="1">
       <c r="A45" s="82" t="s">
-        <v>97</v>
+        <v>79</v>
       </c>
       <c r="B45" s="31"/>
       <c r="C45" s="31"/>
@@ -3736,17 +3739,17 @@
       <c r="H45" s="31"/>
       <c r="I45" s="31"/>
       <c r="J45" s="31"/>
-      <c r="M45" s="155"/>
-      <c r="N45" s="158"/>
-      <c r="O45" s="156"/>
+      <c r="M45" s="154"/>
+      <c r="N45" s="115"/>
+      <c r="O45" s="152"/>
       <c r="P45" s="31"/>
-      <c r="Q45" s="157"/>
-      <c r="R45" s="157"/>
-      <c r="S45" s="157"/>
+      <c r="Q45" s="119"/>
+      <c r="R45" s="119"/>
+      <c r="S45" s="119"/>
     </row>
     <row r="46" spans="1:19" ht="18.75" customHeight="1">
       <c r="A46" s="82" t="s">
-        <v>98</v>
+        <v>80</v>
       </c>
       <c r="B46" s="31"/>
       <c r="C46" s="31"/>
@@ -3766,7 +3769,7 @@
     </row>
     <row r="47" spans="1:19" ht="18.75">
       <c r="A47" s="82" t="s">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="B47" s="31"/>
       <c r="C47" s="31"/>
@@ -3777,24 +3780,24 @@
       <c r="H47" s="31"/>
       <c r="I47" s="31"/>
       <c r="J47" s="31"/>
-      <c r="M47" s="155" t="s">
-        <v>127</v>
+      <c r="M47" s="154" t="s">
+        <v>103</v>
       </c>
       <c r="N47" s="31"/>
-      <c r="O47" s="156" t="e">
+      <c r="O47" s="152" t="e">
         <f>J30+J31-J32</f>
         <v>#REF!</v>
       </c>
       <c r="P47" s="31"/>
-      <c r="Q47" s="157" t="s">
-        <v>128</v>
-      </c>
-      <c r="R47" s="157"/>
-      <c r="S47" s="157"/>
+      <c r="Q47" s="119" t="s">
+        <v>104</v>
+      </c>
+      <c r="R47" s="119"/>
+      <c r="S47" s="119"/>
     </row>
     <row r="48" spans="1:19" ht="18.75">
       <c r="A48" s="82" t="s">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="B48" s="31"/>
       <c r="C48" s="31"/>
@@ -3805,13 +3808,13 @@
       <c r="H48" s="31"/>
       <c r="I48" s="31"/>
       <c r="J48" s="31"/>
-      <c r="M48" s="155"/>
-      <c r="N48" s="158"/>
-      <c r="O48" s="159"/>
+      <c r="M48" s="154"/>
+      <c r="N48" s="115"/>
+      <c r="O48" s="155"/>
       <c r="P48" s="31"/>
-      <c r="Q48" s="157"/>
-      <c r="R48" s="157"/>
-      <c r="S48" s="157"/>
+      <c r="Q48" s="119"/>
+      <c r="R48" s="119"/>
+      <c r="S48" s="119"/>
     </row>
     <row r="49" spans="1:19">
       <c r="A49" s="31"/>
@@ -3832,29 +3835,29 @@
       <c r="S49" s="2"/>
     </row>
     <row r="50" spans="1:19">
-      <c r="M50" s="160" t="s">
-        <v>129</v>
-      </c>
-      <c r="O50" s="161" t="e">
+      <c r="M50" s="116" t="s">
+        <v>105</v>
+      </c>
+      <c r="O50" s="117" t="e">
         <f>J33</f>
         <v>#REF!</v>
       </c>
-      <c r="Q50" s="157" t="s">
-        <v>130</v>
-      </c>
-      <c r="R50" s="157"/>
-      <c r="S50" s="157"/>
+      <c r="Q50" s="119" t="s">
+        <v>106</v>
+      </c>
+      <c r="R50" s="119"/>
+      <c r="S50" s="119"/>
     </row>
     <row r="51" spans="1:19" ht="18.75">
       <c r="H51" s="32"/>
       <c r="I51" s="32"/>
       <c r="J51" s="32"/>
       <c r="K51" s="31"/>
-      <c r="M51" s="160"/>
-      <c r="O51" s="162"/>
-      <c r="Q51" s="157"/>
-      <c r="R51" s="157"/>
-      <c r="S51" s="157"/>
+      <c r="M51" s="116"/>
+      <c r="O51" s="118"/>
+      <c r="Q51" s="119"/>
+      <c r="R51" s="119"/>
+      <c r="S51" s="119"/>
     </row>
     <row r="52" spans="1:19" ht="18.75">
       <c r="H52" s="32"/>
@@ -3868,23 +3871,28 @@
       <c r="J54" s="40"/>
     </row>
     <row r="56" spans="1:19" ht="21">
-      <c r="A56" s="113" t="s">
+      <c r="A56" s="141" t="s">
         <v>45</v>
       </c>
-      <c r="B56" s="113"/>
-      <c r="C56" s="113"/>
-      <c r="D56" s="113"/>
-      <c r="E56" s="113"/>
-      <c r="F56" s="113"/>
-      <c r="G56" s="113"/>
-      <c r="H56" s="113"/>
-      <c r="I56" s="113"/>
-      <c r="J56" s="113"/>
-      <c r="K56" s="113"/>
+      <c r="B56" s="141"/>
+      <c r="C56" s="141"/>
+      <c r="D56" s="141"/>
+      <c r="E56" s="141"/>
+      <c r="F56" s="141"/>
+      <c r="G56" s="141"/>
+      <c r="H56" s="141"/>
+      <c r="I56" s="141"/>
+      <c r="J56" s="141"/>
+      <c r="K56" s="141"/>
+    </row>
+    <row r="59" spans="1:19">
+      <c r="A59" s="1" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="60" spans="1:19">
       <c r="A60" s="49" t="s">
-        <v>47</v>
+        <v>107</v>
       </c>
       <c r="B60" s="31"/>
       <c r="C60" s="31"/>
@@ -3892,7 +3900,7 @@
     </row>
     <row r="61" spans="1:19">
       <c r="A61" s="49" t="s">
-        <v>55</v>
+        <v>108</v>
       </c>
       <c r="B61" s="31"/>
       <c r="C61" s="31"/>
@@ -3900,14 +3908,14 @@
     </row>
     <row r="62" spans="1:19">
       <c r="A62" s="31" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C62" s="31"/>
       <c r="D62" s="31"/>
     </row>
     <row r="63" spans="1:19">
       <c r="A63" s="49" t="s">
-        <v>48</v>
+        <v>109</v>
       </c>
       <c r="B63" s="31"/>
       <c r="C63" s="31"/>
@@ -3915,7 +3923,7 @@
     </row>
     <row r="64" spans="1:19">
       <c r="A64" s="49" t="s">
-        <v>57</v>
+        <v>110</v>
       </c>
       <c r="B64" s="31"/>
       <c r="C64" s="31"/>
@@ -3923,14 +3931,14 @@
     </row>
     <row r="65" spans="1:10">
       <c r="A65" s="31" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="C65" s="31"/>
       <c r="D65" s="31"/>
     </row>
     <row r="66" spans="1:10">
       <c r="A66" s="49" t="s">
-        <v>49</v>
+        <v>111</v>
       </c>
       <c r="B66" s="31"/>
       <c r="C66" s="31"/>
@@ -3938,7 +3946,7 @@
     </row>
     <row r="67" spans="1:10">
       <c r="A67" s="49" t="s">
-        <v>51</v>
+        <v>112</v>
       </c>
       <c r="B67" s="31"/>
       <c r="C67" s="31"/>
@@ -3946,7 +3954,7 @@
     </row>
     <row r="68" spans="1:10">
       <c r="A68" s="49" t="s">
-        <v>58</v>
+        <v>113</v>
       </c>
       <c r="B68" s="31"/>
       <c r="C68" s="31"/>
@@ -3954,7 +3962,7 @@
     </row>
     <row r="69" spans="1:10">
       <c r="A69" s="49" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="B69" s="31"/>
       <c r="C69" s="31"/>
@@ -3962,7 +3970,7 @@
     </row>
     <row r="70" spans="1:10">
       <c r="A70" s="49" t="s">
-        <v>61</v>
+        <v>117</v>
       </c>
       <c r="B70" s="31"/>
       <c r="C70" s="31"/>
@@ -3970,7 +3978,7 @@
     </row>
     <row r="71" spans="1:10">
       <c r="A71" s="49" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="B71" s="31"/>
       <c r="C71" s="31"/>
@@ -3978,7 +3986,7 @@
     </row>
     <row r="72" spans="1:10">
       <c r="A72" s="49" t="s">
-        <v>50</v>
+        <v>114</v>
       </c>
       <c r="B72" s="31"/>
       <c r="C72" s="31"/>
@@ -3986,7 +3994,7 @@
     </row>
     <row r="73" spans="1:10">
       <c r="A73" s="49" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B73" s="31"/>
       <c r="C73" s="31"/>
@@ -3994,7 +4002,7 @@
     </row>
     <row r="77" spans="1:10">
       <c r="A77" s="49" t="s">
-        <v>62</v>
+        <v>118</v>
       </c>
       <c r="B77" s="31"/>
       <c r="C77" s="31"/>
@@ -4008,7 +4016,7 @@
     </row>
     <row r="78" spans="1:10">
       <c r="A78" s="90" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="B78" s="31"/>
       <c r="C78" s="31"/>
@@ -4022,7 +4030,7 @@
     </row>
     <row r="79" spans="1:10">
       <c r="A79" s="49" t="s">
-        <v>63</v>
+        <v>120</v>
       </c>
       <c r="B79" s="31"/>
       <c r="C79" s="31"/>
@@ -4036,7 +4044,7 @@
     </row>
     <row r="80" spans="1:10">
       <c r="A80" s="89" t="s">
-        <v>109</v>
+        <v>90</v>
       </c>
       <c r="C80" s="31"/>
       <c r="D80" s="31"/>
@@ -4049,7 +4057,7 @@
     </row>
     <row r="81" spans="1:10">
       <c r="A81" s="49" t="s">
-        <v>64</v>
+        <v>121</v>
       </c>
       <c r="B81" s="31"/>
       <c r="C81" s="31"/>
@@ -4063,7 +4071,7 @@
     </row>
     <row r="82" spans="1:10">
       <c r="A82" s="35" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C82" s="31"/>
       <c r="D82" s="31"/>
@@ -4076,7 +4084,7 @@
     </row>
     <row r="83" spans="1:10">
       <c r="A83" s="49" t="s">
-        <v>65</v>
+        <v>122</v>
       </c>
       <c r="B83" s="31"/>
       <c r="C83" s="31"/>
@@ -4090,7 +4098,7 @@
     </row>
     <row r="84" spans="1:10">
       <c r="A84" s="49" t="s">
-        <v>66</v>
+        <v>123</v>
       </c>
       <c r="B84" s="31"/>
       <c r="C84" s="31"/>
@@ -4104,7 +4112,7 @@
     </row>
     <row r="85" spans="1:10">
       <c r="A85" s="49" t="s">
-        <v>67</v>
+        <v>124</v>
       </c>
       <c r="B85" s="31"/>
       <c r="C85" s="31"/>
@@ -4118,7 +4126,7 @@
     </row>
     <row r="86" spans="1:10">
       <c r="A86" s="49" t="s">
-        <v>68</v>
+        <v>125</v>
       </c>
       <c r="B86" s="31"/>
       <c r="C86" s="31"/>
@@ -4132,7 +4140,7 @@
     </row>
     <row r="87" spans="1:10">
       <c r="A87" s="49" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="B87" s="31"/>
       <c r="C87" s="31"/>
@@ -4146,7 +4154,7 @@
     </row>
     <row r="91" spans="1:10">
       <c r="A91" s="49" t="s">
-        <v>80</v>
+        <v>127</v>
       </c>
       <c r="B91" s="31"/>
       <c r="C91" s="31"/>
@@ -4154,7 +4162,7 @@
     </row>
     <row r="92" spans="1:10">
       <c r="A92" s="49" t="s">
-        <v>81</v>
+        <v>128</v>
       </c>
       <c r="B92" s="31"/>
       <c r="C92" s="31"/>
@@ -4162,7 +4170,7 @@
     </row>
     <row r="93" spans="1:10">
       <c r="A93" s="41" t="s">
-        <v>112</v>
+        <v>129</v>
       </c>
       <c r="B93" s="31"/>
       <c r="C93" s="31"/>
@@ -4170,12 +4178,12 @@
     </row>
     <row r="94" spans="1:10">
       <c r="A94" s="41" t="s">
-        <v>113</v>
+        <v>130</v>
       </c>
     </row>
     <row r="95" spans="1:10">
       <c r="A95" s="41" t="s">
-        <v>114</v>
+        <v>131</v>
       </c>
     </row>
     <row r="100" spans="2:10">
@@ -4211,6 +4219,23 @@
   </sheetData>
   <sheetProtection selectLockedCells="1"/>
   <mergeCells count="33">
+    <mergeCell ref="O44:O45"/>
+    <mergeCell ref="M39:S40"/>
+    <mergeCell ref="M44:M45"/>
+    <mergeCell ref="Q44:S45"/>
+    <mergeCell ref="M47:M48"/>
+    <mergeCell ref="O47:O48"/>
+    <mergeCell ref="Q47:S48"/>
+    <mergeCell ref="I9:K9"/>
+    <mergeCell ref="A56:K56"/>
+    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="A36:K36"/>
+    <mergeCell ref="B37:D37"/>
+    <mergeCell ref="A29:E29"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="J37:K37"/>
     <mergeCell ref="M50:M51"/>
     <mergeCell ref="O50:O51"/>
     <mergeCell ref="Q50:S51"/>
@@ -4227,23 +4252,6 @@
     <mergeCell ref="I11:K11"/>
     <mergeCell ref="A13:E13"/>
     <mergeCell ref="I8:K8"/>
-    <mergeCell ref="I9:K9"/>
-    <mergeCell ref="A56:K56"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="A36:K36"/>
-    <mergeCell ref="B37:D37"/>
-    <mergeCell ref="A29:E29"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="J37:K37"/>
-    <mergeCell ref="O44:O45"/>
-    <mergeCell ref="M39:S40"/>
-    <mergeCell ref="M44:M45"/>
-    <mergeCell ref="Q44:S45"/>
-    <mergeCell ref="M47:M48"/>
-    <mergeCell ref="O47:O48"/>
-    <mergeCell ref="Q47:S48"/>
   </mergeCells>
   <dataValidations disablePrompts="1" count="2">
     <dataValidation type="custom" showInputMessage="1" showErrorMessage="1" errorTitle="COMPROBAR CANTIDAD DE CAJAS" error="Se debe ingresar la cantidad de cajas" sqref="I11" xr:uid="{3C2F8455-5D0D-41B0-BE98-F91BBC4383D3}">
@@ -4290,19 +4298,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:47" ht="15.75" thickBot="1">
-      <c r="B1" s="145" t="s">
+      <c r="B1" s="156" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="146"/>
-      <c r="D1" s="146"/>
-      <c r="E1" s="146"/>
-      <c r="F1" s="146"/>
-      <c r="G1" s="146"/>
-      <c r="H1" s="146"/>
-      <c r="I1" s="146"/>
-      <c r="J1" s="146"/>
-      <c r="K1" s="146"/>
-      <c r="L1" s="147"/>
+      <c r="C1" s="157"/>
+      <c r="D1" s="157"/>
+      <c r="E1" s="157"/>
+      <c r="F1" s="157"/>
+      <c r="G1" s="157"/>
+      <c r="H1" s="157"/>
+      <c r="I1" s="157"/>
+      <c r="J1" s="157"/>
+      <c r="K1" s="157"/>
+      <c r="L1" s="158"/>
     </row>
     <row r="2" spans="2:47" s="1" customFormat="1" ht="35.1" customHeight="1">
       <c r="B2" s="43"/>
@@ -4321,7 +4329,7 @@
       <c r="B3" s="43"/>
       <c r="C3" s="43"/>
       <c r="D3" s="93" t="s">
-        <v>117</v>
+        <v>93</v>
       </c>
       <c r="E3" s="43"/>
       <c r="F3" s="43"/>
@@ -4334,7 +4342,7 @@
     </row>
     <row r="4" spans="2:47">
       <c r="B4" s="91" t="s">
-        <v>115</v>
+        <v>91</v>
       </c>
       <c r="C4" s="103">
         <v>1</v>
@@ -4366,7 +4374,7 @@
     </row>
     <row r="6" spans="2:47">
       <c r="B6" s="91" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="C6" s="103">
         <v>23.2</v>
@@ -4378,13 +4386,13 @@
     </row>
     <row r="7" spans="2:47">
       <c r="B7" s="91" t="s">
-        <v>72</v>
+        <v>56</v>
       </c>
       <c r="C7" s="103"/>
     </row>
     <row r="8" spans="2:47">
       <c r="B8" s="91" t="s">
-        <v>116</v>
+        <v>92</v>
       </c>
       <c r="C8" s="103">
         <v>8.4000000000000005E-2</v>
@@ -4414,10 +4422,10 @@
     </row>
     <row r="11" spans="2:47" ht="15" customHeight="1">
       <c r="B11" s="87" t="s">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="C11" s="87" t="s">
-        <v>118</v>
+        <v>94</v>
       </c>
       <c r="D11" s="99" t="s">
         <v>8</v>
@@ -4433,7 +4441,7 @@
     </row>
     <row r="12" spans="2:47" ht="15" hidden="1" customHeight="1">
       <c r="B12" s="5" t="s">
-        <v>88</v>
+        <v>70</v>
       </c>
       <c r="C12" s="7"/>
       <c r="D12" s="100">
@@ -4451,7 +4459,7 @@
     </row>
     <row r="13" spans="2:47" ht="15" hidden="1" customHeight="1">
       <c r="B13" s="5" t="s">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="C13" s="86"/>
       <c r="D13" s="101">
@@ -4469,7 +4477,7 @@
     </row>
     <row r="14" spans="2:47" ht="15" hidden="1" customHeight="1">
       <c r="B14" s="5" t="s">
-        <v>82</v>
+        <v>64</v>
       </c>
       <c r="C14" s="85"/>
       <c r="D14" s="102">
@@ -4532,7 +4540,7 @@
     </row>
     <row r="16" spans="2:47" ht="15" hidden="1" customHeight="1">
       <c r="B16" s="54" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="C16" s="55"/>
       <c r="D16" s="1"/>
@@ -4702,7 +4710,7 @@
         <v>#REF!</v>
       </c>
       <c r="E21" s="77"/>
-      <c r="F21" s="149"/>
+      <c r="F21" s="160"/>
       <c r="G21" s="48"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
@@ -4736,7 +4744,7 @@
         <v>#REF!</v>
       </c>
       <c r="E22" s="1"/>
-      <c r="F22" s="149"/>
+      <c r="F22" s="160"/>
       <c r="G22" s="48"/>
       <c r="H22" s="1"/>
       <c r="I22" s="76"/>
@@ -4761,7 +4769,7 @@
     </row>
     <row r="23" spans="2:48" ht="14.25" hidden="1" customHeight="1">
       <c r="B23" s="56" t="s">
-        <v>70</v>
+        <v>54</v>
       </c>
       <c r="C23" s="57" t="e">
         <f>C19+C21</f>
@@ -4855,7 +4863,7 @@
     </row>
     <row r="26" spans="2:48" ht="18.75" hidden="1" customHeight="1">
       <c r="B26" s="56" t="s">
-        <v>71</v>
+        <v>55</v>
       </c>
       <c r="C26" s="57" t="e">
         <f>C23+C24</f>
@@ -4871,19 +4879,19 @@
       <c r="G27" s="48"/>
     </row>
     <row r="28" spans="2:48">
-      <c r="B28" s="151" t="s">
+      <c r="B28" s="162" t="s">
         <v>11</v>
       </c>
-      <c r="C28" s="151"/>
-      <c r="D28" s="151"/>
-      <c r="E28" s="151"/>
-      <c r="F28" s="151"/>
-      <c r="G28" s="151"/>
-      <c r="H28" s="151"/>
-      <c r="I28" s="151"/>
-      <c r="J28" s="151"/>
-      <c r="K28" s="151"/>
-      <c r="L28" s="151"/>
+      <c r="C28" s="162"/>
+      <c r="D28" s="162"/>
+      <c r="E28" s="162"/>
+      <c r="F28" s="162"/>
+      <c r="G28" s="162"/>
+      <c r="H28" s="162"/>
+      <c r="I28" s="162"/>
+      <c r="J28" s="162"/>
+      <c r="K28" s="162"/>
+      <c r="L28" s="162"/>
     </row>
     <row r="30" spans="2:48">
       <c r="C30" s="50"/>
@@ -4918,8 +4926,8 @@
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
       <c r="G33" s="1"/>
-      <c r="H33" s="150"/>
-      <c r="I33" s="150"/>
+      <c r="H33" s="161"/>
+      <c r="I33" s="161"/>
       <c r="J33" s="1"/>
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
@@ -4947,8 +4955,8 @@
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
       <c r="G34" s="1"/>
-      <c r="H34" s="150"/>
-      <c r="I34" s="150"/>
+      <c r="H34" s="161"/>
+      <c r="I34" s="161"/>
       <c r="J34" s="1"/>
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
@@ -5154,19 +5162,19 @@
       </c>
     </row>
     <row r="42" spans="1:47">
-      <c r="B42" s="148" t="s">
+      <c r="B42" s="159" t="s">
         <v>16</v>
       </c>
-      <c r="C42" s="148"/>
-      <c r="D42" s="148"/>
-      <c r="E42" s="148"/>
-      <c r="F42" s="148"/>
-      <c r="G42" s="148"/>
-      <c r="H42" s="148"/>
-      <c r="I42" s="148"/>
-      <c r="J42" s="148"/>
-      <c r="K42" s="148"/>
-      <c r="L42" s="148"/>
+      <c r="C42" s="159"/>
+      <c r="D42" s="159"/>
+      <c r="E42" s="159"/>
+      <c r="F42" s="159"/>
+      <c r="G42" s="159"/>
+      <c r="H42" s="159"/>
+      <c r="I42" s="159"/>
+      <c r="J42" s="159"/>
+      <c r="K42" s="159"/>
+      <c r="L42" s="159"/>
     </row>
     <row r="44" spans="1:47">
       <c r="C44" s="21">

</xml_diff>